<commit_message>
feat(ai): integrate full dual-mode AI support suite (interactive chat desk partner, 1-click trade autopsies, daily EOD debrief, and BYOK Gemini/OpenAI settings)
</commit_message>
<xml_diff>
--- a/deliverables/D3_Tracking_Spreadsheet.xlsx
+++ b/deliverables/D3_Tracking_Spreadsheet.xlsx
@@ -433,10 +433,10 @@
             <c:strLit>
               <c:ptCount val="2"/>
               <c:pt idx="0">
-                <c:v>Wins (50.0%)</c:v>
+                <c:v>Wins (60.0%)</c:v>
               </c:pt>
               <c:pt idx="1">
-                <c:v>Losses (50.0%)</c:v>
+                <c:v>Losses (40.0%)</c:v>
               </c:pt>
             </c:strLit>
           </c:cat>
@@ -444,10 +444,10 @@
             <c:numLit>
               <c:ptCount val="2"/>
               <c:pt idx="0">
-                <c:v>1</c:v>
+                <c:v>3</c:v>
               </c:pt>
               <c:pt idx="1">
-                <c:v>1</c:v>
+                <c:v>2</c:v>
               </c:pt>
             </c:numLit>
           </c:val>
@@ -551,7 +551,7 @@
       <c r="D5" s="13"/>
       <c r="F5" s="14">
         <f>SUM(Trade_Log!U2:U100)</f>
-        <v>9232.16</v>
+        <v>30232.04</v>
       </c>
       <c r="G5" s="14"/>
       <c r="H5" s="14"/>
@@ -599,13 +599,13 @@
     <row r="9" ht="30" customHeight="1">
       <c r="B9" s="18">
         <f>IFERROR(AVERAGE(Trade_Log!V2:V100),0)</f>
-        <v>0.91</v>
+        <v>1.26</v>
       </c>
       <c r="C9" s="18"/>
       <c r="D9" s="18"/>
       <c r="F9" s="15">
         <f>IF(COUNTA(Trade_Log!B2:B100)=0,0,COUNTIF(Trade_Log!W2:W100,"Win")/COUNTA(Trade_Log!B2:B100))</f>
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="G9" s="15"/>
       <c r="H9" s="15"/>
@@ -662,7 +662,7 @@
         <v>20</v>
       </c>
       <c r="G13" s="5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H13" s="3" t="s">
         <v>219</v>
@@ -682,10 +682,10 @@
         <v>25</v>
       </c>
       <c r="G14" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -702,7 +702,7 @@
         <v>35</v>
       </c>
       <c r="G15" s="5">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H15" s="3" t="s">
         <v>36</v>
@@ -719,13 +719,13 @@
         <v>34</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="G16" s="4">
-        <v>687.24</v>
+        <v>1821.66</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
   </sheetData>
@@ -758,7 +758,7 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="17" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="2" ht="28" customHeight="1">
@@ -813,16 +813,16 @@
     </row>
     <row r="3" ht="20">
       <c r="A3" s="5" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B3" s="26" t="s">
         <v>198</v>
       </c>
       <c r="C3" s="26" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="D3" s="26" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E3" s="26" t="s">
         <v>80</v>
@@ -855,24 +855,24 @@
         <v>2.55</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="4" ht="20">
       <c r="A4" s="5" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B4" s="26" t="s">
         <v>198</v>
       </c>
       <c r="C4" s="26" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="D4" s="26" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="E4" s="26" t="s">
         <v>80</v>
@@ -905,10 +905,160 @@
         <v>-0.72</v>
       </c>
       <c r="O4" s="5" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="P4" s="5" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="5" ht="20">
+      <c r="A5" s="5" t="s">
+        <v>233</v>
+      </c>
+      <c r="B5" s="26" t="s">
+        <v>234</v>
+      </c>
+      <c r="C5" s="26" t="s">
+        <v>230</v>
+      </c>
+      <c r="D5" s="26" t="s">
+        <v>235</v>
+      </c>
+      <c r="E5" s="26" t="s">
+        <v>80</v>
+      </c>
+      <c r="F5" s="27">
+        <v>395.55</v>
+      </c>
+      <c r="G5" s="27">
+        <v>393.3</v>
+      </c>
+      <c r="H5" s="27">
+        <v>400.5</v>
+      </c>
+      <c r="I5" s="27">
+        <v>406.2</v>
+      </c>
+      <c r="J5" s="26">
+        <v>2272</v>
+      </c>
+      <c r="K5" s="6">
+        <v>4.73</v>
+      </c>
+      <c r="L5" s="4">
+        <v>368.94</v>
+      </c>
+      <c r="M5" s="4">
+        <v>23827.86</v>
+      </c>
+      <c r="N5" s="19">
+        <v>4.66</v>
+      </c>
+      <c r="O5" s="5" t="s">
         <v>227</v>
+      </c>
+      <c r="P5" s="5" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="6" ht="20">
+      <c r="A6" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="B6" s="26" t="s">
+        <v>234</v>
+      </c>
+      <c r="C6" s="26" t="s">
+        <v>236</v>
+      </c>
+      <c r="D6" s="26" t="s">
+        <v>237</v>
+      </c>
+      <c r="E6" s="26" t="s">
+        <v>80</v>
+      </c>
+      <c r="F6" s="27">
+        <v>1537.1</v>
+      </c>
+      <c r="G6" s="27">
+        <v>1523.8</v>
+      </c>
+      <c r="H6" s="27">
+        <v>1566.36</v>
+      </c>
+      <c r="I6" s="27">
+        <v>1527.8</v>
+      </c>
+      <c r="J6" s="26">
+        <v>625</v>
+      </c>
+      <c r="K6" s="6">
+        <v>0.7</v>
+      </c>
+      <c r="L6" s="4">
+        <v>382.1</v>
+      </c>
+      <c r="M6" s="4">
+        <v>-6194.6</v>
+      </c>
+      <c r="N6" s="19">
+        <v>-0.75</v>
+      </c>
+      <c r="O6" s="5" t="s">
+        <v>232</v>
+      </c>
+      <c r="P6" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="7" ht="20">
+      <c r="A7" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="B7" s="26" t="s">
+        <v>234</v>
+      </c>
+      <c r="C7" s="26" t="s">
+        <v>239</v>
+      </c>
+      <c r="D7" s="26" t="s">
+        <v>237</v>
+      </c>
+      <c r="E7" s="26" t="s">
+        <v>80</v>
+      </c>
+      <c r="F7" s="27">
+        <v>1530.5</v>
+      </c>
+      <c r="G7" s="27">
+        <v>1521.0</v>
+      </c>
+      <c r="H7" s="27">
+        <v>1551.4</v>
+      </c>
+      <c r="I7" s="27">
+        <v>1536.5</v>
+      </c>
+      <c r="J7" s="26">
+        <v>625</v>
+      </c>
+      <c r="K7" s="6">
+        <v>0.63</v>
+      </c>
+      <c r="L7" s="4">
+        <v>383.38</v>
+      </c>
+      <c r="M7" s="4">
+        <v>3366.62</v>
+      </c>
+      <c r="N7" s="19">
+        <v>0.57</v>
+      </c>
+      <c r="O7" s="5" t="s">
+        <v>227</v>
+      </c>
+      <c r="P7" s="5" t="s">
+        <v>238</v>
       </c>
     </row>
   </sheetData>
@@ -1054,19 +1204,19 @@
     </row>
     <row r="2" ht="20">
       <c r="A2" s="5" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>198</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>232</v>
+        <v>240</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>80</v>
@@ -1075,7 +1225,7 @@
         <v>156</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>233</v>
+        <v>241</v>
       </c>
       <c r="I2" s="5" t="s">
         <v>158</v>
@@ -1120,7 +1270,7 @@
         <v>2.55</v>
       </c>
       <c r="W2" s="5" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="X2" s="5">
         <v>5</v>
@@ -1144,27 +1294,27 @@
         <v>158</v>
       </c>
       <c r="AE2" s="0" t="s">
-        <v>234</v>
+        <v>242</v>
       </c>
       <c r="AF2" s="0" t="s">
-        <v>235</v>
+        <v>243</v>
       </c>
     </row>
     <row r="3" ht="20">
       <c r="A3" s="5" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>198</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>232</v>
+        <v>240</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="F3" s="5" t="s">
         <v>80</v>
@@ -1173,7 +1323,7 @@
         <v>156</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>233</v>
+        <v>241</v>
       </c>
       <c r="I3" s="5" t="s">
         <v>158</v>
@@ -1218,7 +1368,7 @@
         <v>-0.72</v>
       </c>
       <c r="W3" s="5" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="X3" s="5">
         <v>5</v>
@@ -1242,10 +1392,304 @@
         <v>158</v>
       </c>
       <c r="AE3" s="0" t="s">
+        <v>244</v>
+      </c>
+      <c r="AF3" s="0" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="4" ht="20">
+      <c r="A4" s="5" t="s">
+        <v>233</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>246</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>230</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>235</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="G4" s="0" t="s">
+        <v>247</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>230</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="L4" s="6">
+        <v>4.73</v>
+      </c>
+      <c r="M4" s="3">
+        <v>0.0256</v>
+      </c>
+      <c r="N4" s="4">
+        <v>5112.0</v>
+      </c>
+      <c r="O4" s="4">
+        <v>395.55</v>
+      </c>
+      <c r="P4" s="4">
+        <v>393.3</v>
+      </c>
+      <c r="Q4" s="4">
+        <v>406.2</v>
+      </c>
+      <c r="R4" s="0">
+        <v>2272</v>
+      </c>
+      <c r="S4" s="4">
+        <v>24196.8</v>
+      </c>
+      <c r="T4" s="4">
+        <v>368.94</v>
+      </c>
+      <c r="U4" s="4">
+        <v>23827.86</v>
+      </c>
+      <c r="V4" s="6">
+        <v>4.66</v>
+      </c>
+      <c r="W4" s="5" t="s">
+        <v>227</v>
+      </c>
+      <c r="X4" s="5">
+        <v>5</v>
+      </c>
+      <c r="Y4" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="Z4" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="AA4" s="5">
+        <v>2</v>
+      </c>
+      <c r="AB4" s="5">
+        <v>2</v>
+      </c>
+      <c r="AC4" s="5">
+        <v>2</v>
+      </c>
+      <c r="AD4" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="AE4" s="0" t="s">
+        <v>248</v>
+      </c>
+      <c r="AF4" s="0" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="5" ht="20">
+      <c r="A5" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>246</v>
+      </c>
+      <c r="D5" s="5" t="s">
         <v>236</v>
       </c>
-      <c r="AF3" s="0" t="s">
+      <c r="E5" s="5" t="s">
         <v>237</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="G5" s="0" t="s">
+        <v>250</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="L5" s="6">
+        <v>0.7</v>
+      </c>
+      <c r="M5" s="3">
+        <v>0.0416</v>
+      </c>
+      <c r="N5" s="4">
+        <v>8312.5</v>
+      </c>
+      <c r="O5" s="4">
+        <v>1537.1</v>
+      </c>
+      <c r="P5" s="4">
+        <v>1523.8</v>
+      </c>
+      <c r="Q5" s="4">
+        <v>1527.8</v>
+      </c>
+      <c r="R5" s="0">
+        <v>625</v>
+      </c>
+      <c r="S5" s="4">
+        <v>-5812.5</v>
+      </c>
+      <c r="T5" s="4">
+        <v>382.1</v>
+      </c>
+      <c r="U5" s="4">
+        <v>-6194.6</v>
+      </c>
+      <c r="V5" s="6">
+        <v>-0.75</v>
+      </c>
+      <c r="W5" s="5" t="s">
+        <v>232</v>
+      </c>
+      <c r="X5" s="5">
+        <v>5</v>
+      </c>
+      <c r="Y5" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="Z5" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="AA5" s="5">
+        <v>6</v>
+      </c>
+      <c r="AB5" s="5">
+        <v>2</v>
+      </c>
+      <c r="AC5" s="5">
+        <v>4</v>
+      </c>
+      <c r="AD5" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="AE5" s="0" t="s">
+        <v>244</v>
+      </c>
+      <c r="AF5" s="0" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="6" ht="20">
+      <c r="A6" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>246</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>239</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="G6" s="0" t="s">
+        <v>252</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>239</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="L6" s="6">
+        <v>0.63</v>
+      </c>
+      <c r="M6" s="3">
+        <v>0.0297</v>
+      </c>
+      <c r="N6" s="4">
+        <v>5937.5</v>
+      </c>
+      <c r="O6" s="4">
+        <v>1530.5</v>
+      </c>
+      <c r="P6" s="4">
+        <v>1521.0</v>
+      </c>
+      <c r="Q6" s="4">
+        <v>1536.5</v>
+      </c>
+      <c r="R6" s="0">
+        <v>625</v>
+      </c>
+      <c r="S6" s="4">
+        <v>3750.0</v>
+      </c>
+      <c r="T6" s="4">
+        <v>383.38</v>
+      </c>
+      <c r="U6" s="4">
+        <v>3366.62</v>
+      </c>
+      <c r="V6" s="6">
+        <v>0.57</v>
+      </c>
+      <c r="W6" s="5" t="s">
+        <v>227</v>
+      </c>
+      <c r="X6" s="5">
+        <v>5</v>
+      </c>
+      <c r="Y6" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="Z6" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="AA6" s="5">
+        <v>2</v>
+      </c>
+      <c r="AB6" s="5">
+        <v>2</v>
+      </c>
+      <c r="AC6" s="5">
+        <v>2</v>
+      </c>
+      <c r="AD6" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="AE6" s="0" t="s">
+        <v>248</v>
+      </c>
+      <c r="AF6" s="0" t="s">
+        <v>251</v>
       </c>
     </row>
   </sheetData>
@@ -1358,7 +1802,51 @@
         <v>159</v>
       </c>
       <c r="N2" s="0" t="s">
-        <v>238</v>
+        <v>253</v>
+      </c>
+    </row>
+    <row r="3" ht="20">
+      <c r="A3" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="B3" s="5">
+        <v>3</v>
+      </c>
+      <c r="C3" s="5">
+        <v>2</v>
+      </c>
+      <c r="D3" s="5">
+        <v>1</v>
+      </c>
+      <c r="E3" s="5">
+        <v>2</v>
+      </c>
+      <c r="F3" s="4">
+        <v>20999.88</v>
+      </c>
+      <c r="G3" s="6">
+        <v>4.48</v>
+      </c>
+      <c r="H3" s="5">
+        <v>3</v>
+      </c>
+      <c r="I3" s="5">
+        <v>0</v>
+      </c>
+      <c r="J3" s="5">
+        <v>5</v>
+      </c>
+      <c r="K3" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="L3" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="M3" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="N3" s="0" t="s">
+        <v>253</v>
       </c>
     </row>
   </sheetData>
@@ -1446,25 +1934,25 @@
         <v>198</v>
       </c>
       <c r="C2" s="5">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D2" s="5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E2" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F2" s="3">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="G2" s="4">
-        <v>9232.16</v>
+        <v>30232.04</v>
       </c>
       <c r="H2" s="6">
-        <v>0.91</v>
+        <v>1.26</v>
       </c>
       <c r="I2" s="6">
-        <v>0.91</v>
+        <v>1.26</v>
       </c>
       <c r="J2" s="3">
         <v>1.0</v>
@@ -1482,10 +1970,10 @@
         <v>160</v>
       </c>
       <c r="O2" s="0" t="s">
-        <v>239</v>
+        <v>254</v>
       </c>
       <c r="P2" s="0" t="s">
-        <v>240</v>
+        <v>255</v>
       </c>
     </row>
   </sheetData>
@@ -1558,19 +2046,19 @@
         <v>198</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="D2" s="0" t="s">
         <v>156</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>241</v>
+        <v>256</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>242</v>
+        <v>257</v>
       </c>
       <c r="G2" s="5">
         <v>2</v>
@@ -1585,13 +2073,13 @@
         <v>159</v>
       </c>
       <c r="K2" s="0" t="s">
+        <v>258</v>
+      </c>
+      <c r="L2" s="0" t="s">
+        <v>259</v>
+      </c>
+      <c r="M2" s="0" t="s">
         <v>243</v>
-      </c>
-      <c r="L2" s="0" t="s">
-        <v>244</v>
-      </c>
-      <c r="M2" s="0" t="s">
-        <v>235</v>
       </c>
     </row>
     <row r="3" ht="20">
@@ -1599,19 +2087,19 @@
         <v>198</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D3" s="0" t="s">
         <v>156</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>241</v>
+        <v>256</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>242</v>
+        <v>257</v>
       </c>
       <c r="G3" s="5">
         <v>2</v>
@@ -1626,13 +2114,136 @@
         <v>159</v>
       </c>
       <c r="K3" s="0" t="s">
-        <v>243</v>
+        <v>258</v>
       </c>
       <c r="L3" s="0" t="s">
-        <v>244</v>
+        <v>259</v>
       </c>
       <c r="M3" s="0" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="4" ht="20">
+      <c r="A4" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>233</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>235</v>
+      </c>
+      <c r="D4" s="0" t="s">
+        <v>247</v>
+      </c>
+      <c r="E4" s="0" t="s">
+        <v>256</v>
+      </c>
+      <c r="F4" s="0" t="s">
+        <v>257</v>
+      </c>
+      <c r="G4" s="5">
+        <v>2</v>
+      </c>
+      <c r="H4" s="5">
+        <v>2</v>
+      </c>
+      <c r="I4" s="5">
+        <v>2</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="K4" s="0" t="s">
+        <v>258</v>
+      </c>
+      <c r="L4" s="0" t="s">
+        <v>259</v>
+      </c>
+      <c r="M4" s="0" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="5" ht="20">
+      <c r="A5" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>237</v>
+      </c>
+      <c r="D5" s="0" t="s">
+        <v>250</v>
+      </c>
+      <c r="E5" s="0" t="s">
+        <v>256</v>
+      </c>
+      <c r="F5" s="0" t="s">
+        <v>257</v>
+      </c>
+      <c r="G5" s="5">
+        <v>6</v>
+      </c>
+      <c r="H5" s="5">
+        <v>2</v>
+      </c>
+      <c r="I5" s="5">
+        <v>4</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="K5" s="0" t="s">
+        <v>258</v>
+      </c>
+      <c r="L5" s="0" t="s">
+        <v>259</v>
+      </c>
+      <c r="M5" s="0" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="6" ht="20">
+      <c r="A6" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="D6" s="0" t="s">
+        <v>252</v>
+      </c>
+      <c r="E6" s="0" t="s">
+        <v>256</v>
+      </c>
+      <c r="F6" s="0" t="s">
+        <v>257</v>
+      </c>
+      <c r="G6" s="5">
+        <v>2</v>
+      </c>
+      <c r="H6" s="5">
+        <v>2</v>
+      </c>
+      <c r="I6" s="5">
+        <v>2</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="K6" s="0" t="s">
+        <v>258</v>
+      </c>
+      <c r="L6" s="0" t="s">
+        <v>259</v>
+      </c>
+      <c r="M6" s="0" t="s">
+        <v>251</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(journal): resolve trade editing and terminal lockout modal conflicts
</commit_message>
<xml_diff>
--- a/deliverables/D3_Tracking_Spreadsheet.xlsx
+++ b/deliverables/D3_Tracking_Spreadsheet.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="184">
   <si>
     <t>TRADER EXECUTION RESET SYSTEM — VISUAL COMMAND CENTER</t>
   </si>
@@ -30,7 +30,7 @@
     <t>CHECKLIST ADHERENCE</t>
   </si>
   <si>
-    <t>₹269,469.57 (+34.73%)</t>
+    <t>₹219,453.82 (+9.73%)</t>
   </si>
   <si>
     <t>Starting Capital: ₹2,00,000 | Risk: ₹500 (0.25%)</t>
@@ -78,7 +78,7 @@
     <t>Wins</t>
   </si>
   <si>
-    <t>71.4%</t>
+    <t>58.3%</t>
   </si>
   <si>
     <t>Minimum Planned RR</t>
@@ -93,7 +93,7 @@
     <t>Losses</t>
   </si>
   <si>
-    <t>28.6%</t>
+    <t>41.7%</t>
   </si>
   <si>
     <t>Broker Kill Switch</t>
@@ -252,6 +252,51 @@
     <t>AGIIL</t>
   </si>
   <si>
+    <t>T-008</t>
+  </si>
+  <si>
+    <t>2026-10-28</t>
+  </si>
+  <si>
+    <t>09:20</t>
+  </si>
+  <si>
+    <t>ONESOURCE</t>
+  </si>
+  <si>
+    <t>T-009</t>
+  </si>
+  <si>
+    <t>11:04</t>
+  </si>
+  <si>
+    <t>T-010</t>
+  </si>
+  <si>
+    <t>13:53</t>
+  </si>
+  <si>
+    <t>ARVIND</t>
+  </si>
+  <si>
+    <t>N (&lt;2.2R)</t>
+  </si>
+  <si>
+    <t>T-011</t>
+  </si>
+  <si>
+    <t>14:29</t>
+  </si>
+  <si>
+    <t>OLAELC</t>
+  </si>
+  <si>
+    <t>T-012</t>
+  </si>
+  <si>
+    <t>15:01</t>
+  </si>
+  <si>
     <t>Day</t>
   </si>
   <si>
@@ -379,6 +424,24 @@
   </si>
   <si>
     <t>https://www.tradingview.com/chart/?symbol=NSE:AGIIL</t>
+  </si>
+  <si>
+    <t>Wed</t>
+  </si>
+  <si>
+    <t>https://www.tradingview.com/chart/?symbol=NSE:ONESOURCE</t>
+  </si>
+  <si>
+    <t>Moved my SL like stupid and took such a big loss, widened the SL and converted small loss to big loss</t>
+  </si>
+  <si>
+    <t>Checklist Incomplete</t>
+  </si>
+  <si>
+    <t>https://www.tradingview.com/chart/?symbol=NSE:ARVIND</t>
+  </si>
+  <si>
+    <t>https://www.tradingview.com/chart/?symbol=NSE:OLAELC</t>
   </si>
   <si>
     <t>Trades_Taken</t>
@@ -923,10 +986,10 @@
             <c:strLit>
               <c:ptCount val="2"/>
               <c:pt idx="0">
-                <c:v>Wins (71.4%)</c:v>
+                <c:v>Wins (58.3%)</c:v>
               </c:pt>
               <c:pt idx="1">
-                <c:v>Losses (28.6%)</c:v>
+                <c:v>Losses (41.7%)</c:v>
               </c:pt>
             </c:strLit>
           </c:cat>
@@ -934,10 +997,10 @@
             <c:numLit>
               <c:ptCount val="2"/>
               <c:pt idx="0">
-                <c:v>5</c:v>
+                <c:v>7</c:v>
               </c:pt>
               <c:pt idx="1">
-                <c:v>2</c:v>
+                <c:v>5</c:v>
               </c:pt>
             </c:numLit>
           </c:val>
@@ -1041,13 +1104,13 @@
       <c r="D5" s="13"/>
       <c r="F5" s="14">
         <f>SUM(Trade_Log!U2:U100)</f>
-        <v>69469.57</v>
+        <v>19453.82</v>
       </c>
       <c r="G5" s="14"/>
       <c r="H5" s="14"/>
       <c r="J5" s="15">
         <f>IF(COUNTA(Trade_Log!B2:B100)=0,0,COUNTIF(Trade_Log!X2:X100,5)/COUNTA(Trade_Log!B2:B100))</f>
-        <v>1.0</v>
+        <v>0.75</v>
       </c>
       <c r="K5" s="15"/>
       <c r="L5" s="15"/>
@@ -1089,19 +1152,19 @@
     <row r="9" ht="30" customHeight="1">
       <c r="B9" s="18">
         <f>IFERROR(AVERAGE(Trade_Log!V2:V100),0)</f>
-        <v>1.9</v>
+        <v>0.45</v>
       </c>
       <c r="C9" s="18"/>
       <c r="D9" s="18"/>
       <c r="F9" s="15">
         <f>IF(COUNTA(Trade_Log!B2:B100)=0,0,COUNTIF(Trade_Log!W2:W100,"Win")/COUNTA(Trade_Log!B2:B100))</f>
-        <v>0.7140000000000001</v>
+        <v>0.583</v>
       </c>
       <c r="G9" s="15"/>
       <c r="H9" s="15"/>
       <c r="J9" s="13">
         <f>COUNTIF(Trade_Log!Y2:Y100,"Y") + COUNTIF(Trade_Log!Z2:Z100,"Revenge")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K9" s="13"/>
       <c r="L9" s="13"/>
@@ -1152,7 +1215,7 @@
         <v>20</v>
       </c>
       <c r="G13" s="5">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H13" s="3" t="s">
         <v>21</v>
@@ -1172,7 +1235,7 @@
         <v>25</v>
       </c>
       <c r="G14" s="5">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H14" s="3" t="s">
         <v>26</v>
@@ -1192,7 +1255,7 @@
         <v>30</v>
       </c>
       <c r="G15" s="5">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="H15" s="3" t="s">
         <v>31</v>
@@ -1212,7 +1275,7 @@
         <v>35</v>
       </c>
       <c r="G16" s="4">
-        <v>2574.58</v>
+        <v>4424.38</v>
       </c>
       <c r="H16" s="3" t="s">
         <v>36</v>
@@ -1649,6 +1712,256 @@
       </c>
       <c r="P9" s="5" t="s">
         <v>60</v>
+      </c>
+    </row>
+    <row r="10" ht="20">
+      <c r="A10" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="B10" s="26" t="s">
+        <v>80</v>
+      </c>
+      <c r="C10" s="26" t="s">
+        <v>81</v>
+      </c>
+      <c r="D10" s="26" t="s">
+        <v>82</v>
+      </c>
+      <c r="E10" s="26" t="s">
+        <v>58</v>
+      </c>
+      <c r="F10" s="27">
+        <v>1624.9</v>
+      </c>
+      <c r="G10" s="27">
+        <v>1610.8</v>
+      </c>
+      <c r="H10" s="27">
+        <v>1655.92</v>
+      </c>
+      <c r="I10" s="27">
+        <v>1626.75</v>
+      </c>
+      <c r="J10" s="26">
+        <v>625</v>
+      </c>
+      <c r="K10" s="6">
+        <v>0.13</v>
+      </c>
+      <c r="L10" s="4">
+        <v>403.31</v>
+      </c>
+      <c r="M10" s="4">
+        <v>752.94</v>
+      </c>
+      <c r="N10" s="19">
+        <v>0.09</v>
+      </c>
+      <c r="O10" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="P10" s="5" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="11" ht="20">
+      <c r="A11" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="B11" s="26" t="s">
+        <v>80</v>
+      </c>
+      <c r="C11" s="26" t="s">
+        <v>84</v>
+      </c>
+      <c r="D11" s="26" t="s">
+        <v>82</v>
+      </c>
+      <c r="E11" s="26" t="s">
+        <v>58</v>
+      </c>
+      <c r="F11" s="27">
+        <v>1633.0</v>
+      </c>
+      <c r="G11" s="27">
+        <v>1621.0</v>
+      </c>
+      <c r="H11" s="27">
+        <v>1659.4</v>
+      </c>
+      <c r="I11" s="27">
+        <v>1562.2</v>
+      </c>
+      <c r="J11" s="26">
+        <v>625</v>
+      </c>
+      <c r="K11" s="6">
+        <v>5.9</v>
+      </c>
+      <c r="L11" s="4">
+        <v>392.14</v>
+      </c>
+      <c r="M11" s="4">
+        <v>-44642.14</v>
+      </c>
+      <c r="N11" s="19">
+        <v>-5.95</v>
+      </c>
+      <c r="O11" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="P11" s="5" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="12" ht="20">
+      <c r="A12" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="B12" s="26" t="s">
+        <v>80</v>
+      </c>
+      <c r="C12" s="26" t="s">
+        <v>86</v>
+      </c>
+      <c r="D12" s="26" t="s">
+        <v>87</v>
+      </c>
+      <c r="E12" s="26" t="s">
+        <v>58</v>
+      </c>
+      <c r="F12" s="27">
+        <v>523.0</v>
+      </c>
+      <c r="G12" s="27">
+        <v>520.0</v>
+      </c>
+      <c r="H12" s="27">
+        <v>529.6</v>
+      </c>
+      <c r="I12" s="27">
+        <v>517.0</v>
+      </c>
+      <c r="J12" s="26">
+        <v>1639</v>
+      </c>
+      <c r="K12" s="6">
+        <v>2.0</v>
+      </c>
+      <c r="L12" s="4">
+        <v>344.7</v>
+      </c>
+      <c r="M12" s="4">
+        <v>-10178.7</v>
+      </c>
+      <c r="N12" s="19">
+        <v>-2.07</v>
+      </c>
+      <c r="O12" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="P12" s="5" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="13" ht="20">
+      <c r="A13" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="B13" s="26" t="s">
+        <v>80</v>
+      </c>
+      <c r="C13" s="26" t="s">
+        <v>90</v>
+      </c>
+      <c r="D13" s="26" t="s">
+        <v>91</v>
+      </c>
+      <c r="E13" s="26" t="s">
+        <v>58</v>
+      </c>
+      <c r="F13" s="27">
+        <v>36.9</v>
+      </c>
+      <c r="G13" s="27">
+        <v>36.35</v>
+      </c>
+      <c r="H13" s="27">
+        <v>38.11</v>
+      </c>
+      <c r="I13" s="27">
+        <v>37.2</v>
+      </c>
+      <c r="J13" s="26">
+        <v>23809</v>
+      </c>
+      <c r="K13" s="6">
+        <v>0.55</v>
+      </c>
+      <c r="L13" s="4">
+        <v>357.02</v>
+      </c>
+      <c r="M13" s="4">
+        <v>6785.68</v>
+      </c>
+      <c r="N13" s="19">
+        <v>0.52</v>
+      </c>
+      <c r="O13" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="P13" s="5" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="14" ht="20">
+      <c r="A14" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="B14" s="26" t="s">
+        <v>80</v>
+      </c>
+      <c r="C14" s="26" t="s">
+        <v>93</v>
+      </c>
+      <c r="D14" s="26" t="s">
+        <v>91</v>
+      </c>
+      <c r="E14" s="26" t="s">
+        <v>58</v>
+      </c>
+      <c r="F14" s="27">
+        <v>36.7</v>
+      </c>
+      <c r="G14" s="27">
+        <v>36.5</v>
+      </c>
+      <c r="H14" s="27">
+        <v>37.14</v>
+      </c>
+      <c r="I14" s="27">
+        <v>36.6</v>
+      </c>
+      <c r="J14" s="26">
+        <v>23809</v>
+      </c>
+      <c r="K14" s="6">
+        <v>0.5</v>
+      </c>
+      <c r="L14" s="4">
+        <v>352.63</v>
+      </c>
+      <c r="M14" s="4">
+        <v>-2733.53</v>
+      </c>
+      <c r="N14" s="19">
+        <v>-0.57</v>
+      </c>
+      <c r="O14" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="P14" s="5" t="s">
+        <v>88</v>
       </c>
     </row>
   </sheetData>
@@ -1702,10 +2015,10 @@
         <v>39</v>
       </c>
       <c r="C1" s="25" t="s">
-        <v>79</v>
+        <v>94</v>
       </c>
       <c r="D1" s="24" t="s">
-        <v>80</v>
+        <v>95</v>
       </c>
       <c r="E1" s="24" t="s">
         <v>41</v>
@@ -1714,28 +2027,28 @@
         <v>42</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>81</v>
+        <v>96</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>82</v>
+        <v>97</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>85</v>
+        <v>100</v>
       </c>
       <c r="L1" s="25" t="s">
-        <v>86</v>
+        <v>101</v>
       </c>
       <c r="M1" s="25" t="s">
-        <v>87</v>
+        <v>102</v>
       </c>
       <c r="N1" s="25" t="s">
-        <v>88</v>
+        <v>103</v>
       </c>
       <c r="O1" s="24" t="s">
         <v>43</v>
@@ -1750,46 +2063,46 @@
         <v>47</v>
       </c>
       <c r="S1" s="25" t="s">
-        <v>89</v>
+        <v>104</v>
       </c>
       <c r="T1" s="25" t="s">
-        <v>90</v>
+        <v>105</v>
       </c>
       <c r="U1" s="25" t="s">
         <v>50</v>
       </c>
       <c r="V1" s="25" t="s">
-        <v>91</v>
+        <v>106</v>
       </c>
       <c r="W1" s="25" t="s">
         <v>52</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>92</v>
+        <v>107</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>93</v>
+        <v>108</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>94</v>
+        <v>109</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>95</v>
+        <v>110</v>
       </c>
       <c r="AB1" s="1" t="s">
-        <v>96</v>
+        <v>111</v>
       </c>
       <c r="AC1" s="1" t="s">
-        <v>97</v>
+        <v>112</v>
       </c>
       <c r="AD1" s="25" t="s">
-        <v>98</v>
+        <v>113</v>
       </c>
       <c r="AE1" s="1" t="s">
-        <v>99</v>
+        <v>114</v>
       </c>
       <c r="AF1" s="1" t="s">
-        <v>100</v>
+        <v>115</v>
       </c>
     </row>
     <row r="2" ht="20">
@@ -1800,7 +2113,7 @@
         <v>55</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>101</v>
+        <v>116</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>56</v>
@@ -1812,19 +2125,19 @@
         <v>58</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>103</v>
+        <v>118</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="L2" s="6">
         <v>2.2</v>
@@ -1866,10 +2179,10 @@
         <v>5</v>
       </c>
       <c r="Y2" s="5" t="s">
-        <v>105</v>
+        <v>120</v>
       </c>
       <c r="Z2" s="5" t="s">
-        <v>106</v>
+        <v>121</v>
       </c>
       <c r="AA2" s="5">
         <v>2</v>
@@ -1881,13 +2194,13 @@
         <v>2</v>
       </c>
       <c r="AD2" s="5" t="s">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="AE2" s="0" t="s">
-        <v>107</v>
+        <v>122</v>
       </c>
       <c r="AF2" s="0" t="s">
-        <v>108</v>
+        <v>123</v>
       </c>
     </row>
     <row r="3" ht="20">
@@ -1898,7 +2211,7 @@
         <v>55</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>101</v>
+        <v>116</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>62</v>
@@ -1910,19 +2223,19 @@
         <v>58</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>103</v>
+        <v>118</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="L3" s="6">
         <v>2.2</v>
@@ -1964,10 +2277,10 @@
         <v>5</v>
       </c>
       <c r="Y3" s="5" t="s">
-        <v>105</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="5" t="s">
-        <v>106</v>
+        <v>121</v>
       </c>
       <c r="AA3" s="5">
         <v>2</v>
@@ -1979,13 +2292,13 @@
         <v>2</v>
       </c>
       <c r="AD3" s="5" t="s">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="AE3" s="0" t="s">
-        <v>109</v>
+        <v>124</v>
       </c>
       <c r="AF3" s="0" t="s">
-        <v>110</v>
+        <v>125</v>
       </c>
     </row>
     <row r="4" ht="20">
@@ -1996,7 +2309,7 @@
         <v>66</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>111</v>
+        <v>126</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>62</v>
@@ -2008,19 +2321,19 @@
         <v>58</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>112</v>
+        <v>127</v>
       </c>
       <c r="H4" s="5" t="s">
         <v>62</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="L4" s="6">
         <v>4.73</v>
@@ -2062,10 +2375,10 @@
         <v>5</v>
       </c>
       <c r="Y4" s="5" t="s">
-        <v>105</v>
+        <v>120</v>
       </c>
       <c r="Z4" s="5" t="s">
-        <v>106</v>
+        <v>121</v>
       </c>
       <c r="AA4" s="5">
         <v>2</v>
@@ -2077,13 +2390,13 @@
         <v>2</v>
       </c>
       <c r="AD4" s="5" t="s">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="AE4" s="0" t="s">
-        <v>113</v>
+        <v>128</v>
       </c>
       <c r="AF4" s="0" t="s">
-        <v>114</v>
+        <v>129</v>
       </c>
     </row>
     <row r="5" ht="20">
@@ -2094,7 +2407,7 @@
         <v>66</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>111</v>
+        <v>126</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>69</v>
@@ -2106,19 +2419,19 @@
         <v>58</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>115</v>
+        <v>130</v>
       </c>
       <c r="H5" s="5" t="s">
         <v>69</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="L5" s="6">
         <v>0.7</v>
@@ -2160,10 +2473,10 @@
         <v>5</v>
       </c>
       <c r="Y5" s="5" t="s">
-        <v>105</v>
+        <v>120</v>
       </c>
       <c r="Z5" s="5" t="s">
-        <v>106</v>
+        <v>121</v>
       </c>
       <c r="AA5" s="5">
         <v>6</v>
@@ -2175,13 +2488,13 @@
         <v>4</v>
       </c>
       <c r="AD5" s="5" t="s">
-        <v>105</v>
+        <v>120</v>
       </c>
       <c r="AE5" s="0" t="s">
-        <v>109</v>
+        <v>124</v>
       </c>
       <c r="AF5" s="0" t="s">
-        <v>116</v>
+        <v>131</v>
       </c>
     </row>
     <row r="6" ht="20">
@@ -2192,7 +2505,7 @@
         <v>66</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>111</v>
+        <v>126</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>72</v>
@@ -2204,19 +2517,19 @@
         <v>58</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>117</v>
+        <v>132</v>
       </c>
       <c r="H6" s="5" t="s">
         <v>72</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="L6" s="6">
         <v>0.63</v>
@@ -2258,10 +2571,10 @@
         <v>5</v>
       </c>
       <c r="Y6" s="5" t="s">
-        <v>105</v>
+        <v>120</v>
       </c>
       <c r="Z6" s="5" t="s">
-        <v>106</v>
+        <v>121</v>
       </c>
       <c r="AA6" s="5">
         <v>2</v>
@@ -2273,13 +2586,13 @@
         <v>2</v>
       </c>
       <c r="AD6" s="5" t="s">
-        <v>105</v>
+        <v>120</v>
       </c>
       <c r="AE6" s="0" t="s">
-        <v>113</v>
+        <v>128</v>
       </c>
       <c r="AF6" s="0" t="s">
-        <v>116</v>
+        <v>131</v>
       </c>
     </row>
     <row r="7" ht="20">
@@ -2290,7 +2603,7 @@
         <v>74</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>118</v>
+        <v>133</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>62</v>
@@ -2302,19 +2615,19 @@
         <v>58</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>112</v>
+        <v>127</v>
       </c>
       <c r="H7" s="5" t="s">
         <v>62</v>
       </c>
       <c r="I7" s="5" t="s">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="J7" s="5" t="s">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="K7" s="5" t="s">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="L7" s="6">
         <v>3.11</v>
@@ -2356,10 +2669,10 @@
         <v>5</v>
       </c>
       <c r="Y7" s="5" t="s">
-        <v>105</v>
+        <v>120</v>
       </c>
       <c r="Z7" s="5" t="s">
-        <v>106</v>
+        <v>121</v>
       </c>
       <c r="AA7" s="5">
         <v>3</v>
@@ -2371,13 +2684,13 @@
         <v>2</v>
       </c>
       <c r="AD7" s="5" t="s">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="AE7" s="0" t="s">
-        <v>113</v>
+        <v>128</v>
       </c>
       <c r="AF7" s="0" t="s">
-        <v>119</v>
+        <v>134</v>
       </c>
     </row>
     <row r="8" ht="20">
@@ -2388,7 +2701,7 @@
         <v>74</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>118</v>
+        <v>133</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>77</v>
@@ -2400,19 +2713,19 @@
         <v>58</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>120</v>
+        <v>135</v>
       </c>
       <c r="H8" s="5" t="s">
         <v>77</v>
       </c>
       <c r="I8" s="5" t="s">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="J8" s="5" t="s">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="K8" s="5" t="s">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="L8" s="6">
         <v>4.03</v>
@@ -2454,10 +2767,10 @@
         <v>5</v>
       </c>
       <c r="Y8" s="5" t="s">
-        <v>105</v>
+        <v>120</v>
       </c>
       <c r="Z8" s="5" t="s">
-        <v>106</v>
+        <v>121</v>
       </c>
       <c r="AA8" s="5">
         <v>2</v>
@@ -2469,13 +2782,503 @@
         <v>2</v>
       </c>
       <c r="AD8" s="5" t="s">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="AE8" s="0" t="s">
-        <v>113</v>
+        <v>128</v>
       </c>
       <c r="AF8" s="0" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="9" ht="20">
+      <c r="A9" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="G9" s="0" t="s">
+        <v>135</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="I9" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="J9" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="K9" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="L9" s="6">
+        <v>0.13</v>
+      </c>
+      <c r="M9" s="3">
+        <v>0.0441</v>
+      </c>
+      <c r="N9" s="4">
+        <v>8812.5</v>
+      </c>
+      <c r="O9" s="4">
+        <v>1624.9</v>
+      </c>
+      <c r="P9" s="4">
+        <v>1610.8</v>
+      </c>
+      <c r="Q9" s="4">
+        <v>1626.75</v>
+      </c>
+      <c r="R9" s="0">
+        <v>625</v>
+      </c>
+      <c r="S9" s="4">
+        <v>1156.25</v>
+      </c>
+      <c r="T9" s="4">
+        <v>403.31</v>
+      </c>
+      <c r="U9" s="4">
+        <v>752.94</v>
+      </c>
+      <c r="V9" s="6">
+        <v>0.09</v>
+      </c>
+      <c r="W9" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="X9" s="5">
+        <v>5</v>
+      </c>
+      <c r="Y9" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="Z9" s="5" t="s">
         <v>121</v>
+      </c>
+      <c r="AA9" s="5">
+        <v>3</v>
+      </c>
+      <c r="AB9" s="5">
+        <v>2</v>
+      </c>
+      <c r="AC9" s="5">
+        <v>2</v>
+      </c>
+      <c r="AD9" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="AE9" s="0" t="s">
+        <v>128</v>
+      </c>
+      <c r="AF9" s="0" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="10" ht="20">
+      <c r="A10" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="G10" s="0" t="s">
+        <v>117</v>
+      </c>
+      <c r="H10" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="I10" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="J10" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="K10" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="L10" s="6">
+        <v>5.9</v>
+      </c>
+      <c r="M10" s="3">
+        <v>0.0375</v>
+      </c>
+      <c r="N10" s="4">
+        <v>7500.0</v>
+      </c>
+      <c r="O10" s="4">
+        <v>1633.0</v>
+      </c>
+      <c r="P10" s="4">
+        <v>1621.0</v>
+      </c>
+      <c r="Q10" s="4">
+        <v>1562.2</v>
+      </c>
+      <c r="R10" s="0">
+        <v>625</v>
+      </c>
+      <c r="S10" s="4">
+        <v>-44250.0</v>
+      </c>
+      <c r="T10" s="4">
+        <v>392.14</v>
+      </c>
+      <c r="U10" s="4">
+        <v>-44642.14</v>
+      </c>
+      <c r="V10" s="6">
+        <v>-5.95</v>
+      </c>
+      <c r="W10" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="X10" s="5">
+        <v>5</v>
+      </c>
+      <c r="Y10" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="Z10" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="AA10" s="5">
+        <v>3</v>
+      </c>
+      <c r="AB10" s="5">
+        <v>2</v>
+      </c>
+      <c r="AC10" s="5">
+        <v>4</v>
+      </c>
+      <c r="AD10" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="AE10" s="0" t="s">
+        <v>139</v>
+      </c>
+      <c r="AF10" s="0" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="11" ht="20">
+      <c r="A11" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="G11" s="0" t="s">
+        <v>132</v>
+      </c>
+      <c r="H11" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="I11" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="J11" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="K11" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="L11" s="6">
+        <v>2.0</v>
+      </c>
+      <c r="M11" s="3">
+        <v>0.0246</v>
+      </c>
+      <c r="N11" s="4">
+        <v>4917.0</v>
+      </c>
+      <c r="O11" s="4">
+        <v>523.0</v>
+      </c>
+      <c r="P11" s="4">
+        <v>520.0</v>
+      </c>
+      <c r="Q11" s="4">
+        <v>517.0</v>
+      </c>
+      <c r="R11" s="0">
+        <v>1639</v>
+      </c>
+      <c r="S11" s="4">
+        <v>-9834.0</v>
+      </c>
+      <c r="T11" s="4">
+        <v>344.7</v>
+      </c>
+      <c r="U11" s="4">
+        <v>-10178.7</v>
+      </c>
+      <c r="V11" s="6">
+        <v>-2.07</v>
+      </c>
+      <c r="W11" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="X11" s="5">
+        <v>1</v>
+      </c>
+      <c r="Y11" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="Z11" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="AA11" s="5">
+        <v>2</v>
+      </c>
+      <c r="AB11" s="5">
+        <v>2</v>
+      </c>
+      <c r="AC11" s="5">
+        <v>4</v>
+      </c>
+      <c r="AD11" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="AE11" s="0" t="s">
+        <v>124</v>
+      </c>
+      <c r="AF11" s="0" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="12" ht="20">
+      <c r="A12" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="G12" s="0" t="s">
+        <v>132</v>
+      </c>
+      <c r="H12" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="I12" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="J12" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="K12" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="L12" s="6">
+        <v>0.55</v>
+      </c>
+      <c r="M12" s="3">
+        <v>0.0655</v>
+      </c>
+      <c r="N12" s="4">
+        <v>13094.95</v>
+      </c>
+      <c r="O12" s="4">
+        <v>36.9</v>
+      </c>
+      <c r="P12" s="4">
+        <v>36.35</v>
+      </c>
+      <c r="Q12" s="4">
+        <v>37.2</v>
+      </c>
+      <c r="R12" s="0">
+        <v>23809</v>
+      </c>
+      <c r="S12" s="4">
+        <v>7142.7</v>
+      </c>
+      <c r="T12" s="4">
+        <v>357.02</v>
+      </c>
+      <c r="U12" s="4">
+        <v>6785.68</v>
+      </c>
+      <c r="V12" s="6">
+        <v>0.52</v>
+      </c>
+      <c r="W12" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="X12" s="5">
+        <v>1</v>
+      </c>
+      <c r="Y12" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="Z12" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="AA12" s="5">
+        <v>2</v>
+      </c>
+      <c r="AB12" s="5">
+        <v>2</v>
+      </c>
+      <c r="AC12" s="5">
+        <v>2</v>
+      </c>
+      <c r="AD12" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="AE12" s="0" t="s">
+        <v>128</v>
+      </c>
+      <c r="AF12" s="0" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="13" ht="20">
+      <c r="A13" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="G13" s="0" t="s">
+        <v>132</v>
+      </c>
+      <c r="H13" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="I13" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="J13" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="K13" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="L13" s="6">
+        <v>0.5</v>
+      </c>
+      <c r="M13" s="3">
+        <v>0.0238</v>
+      </c>
+      <c r="N13" s="4">
+        <v>4761.8</v>
+      </c>
+      <c r="O13" s="4">
+        <v>36.7</v>
+      </c>
+      <c r="P13" s="4">
+        <v>36.5</v>
+      </c>
+      <c r="Q13" s="4">
+        <v>36.6</v>
+      </c>
+      <c r="R13" s="0">
+        <v>23809</v>
+      </c>
+      <c r="S13" s="4">
+        <v>-2380.9</v>
+      </c>
+      <c r="T13" s="4">
+        <v>352.63</v>
+      </c>
+      <c r="U13" s="4">
+        <v>-2733.53</v>
+      </c>
+      <c r="V13" s="6">
+        <v>-0.57</v>
+      </c>
+      <c r="W13" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="X13" s="5">
+        <v>5</v>
+      </c>
+      <c r="Y13" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="Z13" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="AA13" s="5">
+        <v>2</v>
+      </c>
+      <c r="AB13" s="5">
+        <v>2</v>
+      </c>
+      <c r="AC13" s="5">
+        <v>4</v>
+      </c>
+      <c r="AD13" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="AE13" s="0" t="s">
+        <v>124</v>
+      </c>
+      <c r="AF13" s="0" t="s">
+        <v>142</v>
       </c>
     </row>
   </sheetData>
@@ -2508,43 +3311,43 @@
         <v>39</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>122</v>
+        <v>143</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>123</v>
+        <v>144</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>25</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>124</v>
+        <v>145</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>126</v>
+        <v>147</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>127</v>
+        <v>148</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>128</v>
+        <v>149</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>129</v>
+        <v>150</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>130</v>
+        <v>151</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>131</v>
+        <v>152</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>132</v>
+        <v>153</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>133</v>
+        <v>154</v>
       </c>
     </row>
     <row r="2" ht="20">
@@ -2582,13 +3385,13 @@
         <v>1.0</v>
       </c>
       <c r="L2" s="5" t="s">
-        <v>105</v>
+        <v>120</v>
       </c>
       <c r="M2" s="5" t="s">
-        <v>105</v>
+        <v>120</v>
       </c>
       <c r="N2" s="0" t="s">
-        <v>134</v>
+        <v>155</v>
       </c>
     </row>
     <row r="3" ht="20">
@@ -2626,13 +3429,13 @@
         <v>1.0</v>
       </c>
       <c r="L3" s="5" t="s">
-        <v>105</v>
+        <v>120</v>
       </c>
       <c r="M3" s="5" t="s">
-        <v>105</v>
+        <v>120</v>
       </c>
       <c r="N3" s="0" t="s">
-        <v>134</v>
+        <v>155</v>
       </c>
     </row>
     <row r="4" ht="20">
@@ -2670,13 +3473,57 @@
         <v>1.0</v>
       </c>
       <c r="L4" s="5" t="s">
-        <v>105</v>
+        <v>120</v>
       </c>
       <c r="M4" s="5" t="s">
-        <v>105</v>
+        <v>120</v>
       </c>
       <c r="N4" s="0" t="s">
-        <v>134</v>
+        <v>155</v>
+      </c>
+    </row>
+    <row r="5" ht="20">
+      <c r="A5" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B5" s="5">
+        <v>5</v>
+      </c>
+      <c r="C5" s="5">
+        <v>2</v>
+      </c>
+      <c r="D5" s="5">
+        <v>3</v>
+      </c>
+      <c r="E5" s="5">
+        <v>2</v>
+      </c>
+      <c r="F5" s="4">
+        <v>-50015.75</v>
+      </c>
+      <c r="G5" s="6">
+        <v>-7.98</v>
+      </c>
+      <c r="H5" s="5">
+        <v>3</v>
+      </c>
+      <c r="I5" s="5">
+        <v>3</v>
+      </c>
+      <c r="J5" s="5">
+        <v>5</v>
+      </c>
+      <c r="K5" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="L5" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="M5" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="N5" s="0" t="s">
+        <v>155</v>
       </c>
     </row>
   </sheetData>
@@ -2708,13 +3555,13 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>135</v>
+        <v>156</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>136</v>
+        <v>157</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>137</v>
+        <v>158</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>20</v>
@@ -2723,87 +3570,87 @@
         <v>25</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>138</v>
+        <v>159</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>50</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>139</v>
+        <v>160</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>140</v>
+        <v>161</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>142</v>
+        <v>163</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>143</v>
+        <v>164</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>144</v>
+        <v>165</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>145</v>
+        <v>166</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>146</v>
+        <v>167</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>147</v>
+        <v>168</v>
       </c>
     </row>
     <row r="2" ht="20">
       <c r="A2" s="2" t="s">
-        <v>148</v>
+        <v>169</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>55</v>
       </c>
       <c r="C2" s="5">
+        <v>12</v>
+      </c>
+      <c r="D2" s="5">
         <v>7</v>
       </c>
-      <c r="D2" s="5">
+      <c r="E2" s="5">
         <v>5</v>
       </c>
-      <c r="E2" s="5">
-        <v>2</v>
-      </c>
       <c r="F2" s="3">
-        <v>0.7140000000000001</v>
+        <v>0.583</v>
       </c>
       <c r="G2" s="4">
-        <v>69469.57</v>
+        <v>19453.82</v>
       </c>
       <c r="H2" s="6">
-        <v>1.9</v>
+        <v>0.45</v>
       </c>
       <c r="I2" s="6">
-        <v>1.9</v>
+        <v>0.45</v>
       </c>
       <c r="J2" s="3">
-        <v>1.0</v>
+        <v>0.75</v>
       </c>
       <c r="K2" s="5">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L2" s="5">
         <v>0</v>
       </c>
       <c r="M2" s="5" t="s">
-        <v>149</v>
+        <v>170</v>
       </c>
       <c r="N2" s="5" t="s">
-        <v>106</v>
+        <v>121</v>
       </c>
       <c r="O2" s="0" t="s">
-        <v>150</v>
+        <v>171</v>
       </c>
       <c r="P2" s="0" t="s">
-        <v>151</v>
+        <v>172</v>
       </c>
     </row>
   </sheetData>
@@ -2841,34 +3688,34 @@
         <v>41</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>152</v>
+        <v>173</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>153</v>
+        <v>174</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>154</v>
+        <v>175</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>155</v>
+        <v>176</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>156</v>
+        <v>177</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>157</v>
+        <v>178</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>93</v>
+        <v>108</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>158</v>
+        <v>179</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>159</v>
+        <v>180</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>100</v>
+        <v>115</v>
       </c>
     </row>
     <row r="2" ht="20">
@@ -2882,13 +3729,13 @@
         <v>57</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>160</v>
+        <v>181</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>161</v>
+        <v>182</v>
       </c>
       <c r="G2" s="5">
         <v>2</v>
@@ -2900,16 +3747,16 @@
         <v>2</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>105</v>
+        <v>120</v>
       </c>
       <c r="K2" s="0" t="s">
-        <v>107</v>
+        <v>122</v>
       </c>
       <c r="L2" s="0" t="s">
-        <v>162</v>
+        <v>183</v>
       </c>
       <c r="M2" s="0" t="s">
-        <v>108</v>
+        <v>123</v>
       </c>
     </row>
     <row r="3" ht="20">
@@ -2923,13 +3770,13 @@
         <v>63</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>160</v>
+        <v>181</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>161</v>
+        <v>182</v>
       </c>
       <c r="G3" s="5">
         <v>2</v>
@@ -2941,16 +3788,16 @@
         <v>2</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>105</v>
+        <v>120</v>
       </c>
       <c r="K3" s="0" t="s">
-        <v>109</v>
+        <v>124</v>
       </c>
       <c r="L3" s="0" t="s">
-        <v>162</v>
+        <v>183</v>
       </c>
       <c r="M3" s="0" t="s">
-        <v>110</v>
+        <v>125</v>
       </c>
     </row>
     <row r="4" ht="20">
@@ -2964,13 +3811,13 @@
         <v>67</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>112</v>
+        <v>127</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>160</v>
+        <v>181</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>161</v>
+        <v>182</v>
       </c>
       <c r="G4" s="5">
         <v>2</v>
@@ -2982,16 +3829,16 @@
         <v>2</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>105</v>
+        <v>120</v>
       </c>
       <c r="K4" s="0" t="s">
-        <v>113</v>
+        <v>128</v>
       </c>
       <c r="L4" s="0" t="s">
-        <v>162</v>
+        <v>183</v>
       </c>
       <c r="M4" s="0" t="s">
-        <v>114</v>
+        <v>129</v>
       </c>
     </row>
     <row r="5" ht="20">
@@ -3005,13 +3852,13 @@
         <v>70</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>115</v>
+        <v>130</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>160</v>
+        <v>181</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>161</v>
+        <v>182</v>
       </c>
       <c r="G5" s="5">
         <v>6</v>
@@ -3023,16 +3870,16 @@
         <v>4</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>105</v>
+        <v>120</v>
       </c>
       <c r="K5" s="0" t="s">
-        <v>109</v>
+        <v>124</v>
       </c>
       <c r="L5" s="0" t="s">
-        <v>162</v>
+        <v>183</v>
       </c>
       <c r="M5" s="0" t="s">
-        <v>116</v>
+        <v>131</v>
       </c>
     </row>
     <row r="6" ht="20">
@@ -3046,13 +3893,13 @@
         <v>70</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>117</v>
+        <v>132</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>160</v>
+        <v>181</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>161</v>
+        <v>182</v>
       </c>
       <c r="G6" s="5">
         <v>2</v>
@@ -3064,16 +3911,16 @@
         <v>2</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>105</v>
+        <v>120</v>
       </c>
       <c r="K6" s="0" t="s">
-        <v>113</v>
+        <v>128</v>
       </c>
       <c r="L6" s="0" t="s">
-        <v>162</v>
+        <v>183</v>
       </c>
       <c r="M6" s="0" t="s">
-        <v>116</v>
+        <v>131</v>
       </c>
     </row>
     <row r="7" ht="20">
@@ -3087,13 +3934,13 @@
         <v>75</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>112</v>
+        <v>127</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>160</v>
+        <v>181</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>161</v>
+        <v>182</v>
       </c>
       <c r="G7" s="5">
         <v>3</v>
@@ -3105,16 +3952,16 @@
         <v>2</v>
       </c>
       <c r="J7" s="5" t="s">
-        <v>105</v>
+        <v>120</v>
       </c>
       <c r="K7" s="0" t="s">
-        <v>113</v>
+        <v>128</v>
       </c>
       <c r="L7" s="0" t="s">
-        <v>162</v>
+        <v>183</v>
       </c>
       <c r="M7" s="0" t="s">
-        <v>119</v>
+        <v>134</v>
       </c>
     </row>
     <row r="8" ht="20">
@@ -3128,34 +3975,239 @@
         <v>78</v>
       </c>
       <c r="D8" s="0" t="s">
+        <v>135</v>
+      </c>
+      <c r="E8" s="0" t="s">
+        <v>181</v>
+      </c>
+      <c r="F8" s="0" t="s">
+        <v>182</v>
+      </c>
+      <c r="G8" s="5">
+        <v>2</v>
+      </c>
+      <c r="H8" s="5">
+        <v>2</v>
+      </c>
+      <c r="I8" s="5">
+        <v>2</v>
+      </c>
+      <c r="J8" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="E8" s="0" t="s">
-        <v>160</v>
-      </c>
-      <c r="F8" s="0" t="s">
-        <v>161</v>
-      </c>
-      <c r="G8" s="5">
-        <v>2</v>
-      </c>
-      <c r="H8" s="5">
-        <v>2</v>
-      </c>
-      <c r="I8" s="5">
-        <v>2</v>
-      </c>
-      <c r="J8" s="5" t="s">
-        <v>105</v>
-      </c>
       <c r="K8" s="0" t="s">
-        <v>113</v>
+        <v>128</v>
       </c>
       <c r="L8" s="0" t="s">
-        <v>162</v>
+        <v>183</v>
       </c>
       <c r="M8" s="0" t="s">
-        <v>121</v>
+        <v>136</v>
+      </c>
+    </row>
+    <row r="9" ht="20">
+      <c r="A9" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="D9" s="0" t="s">
+        <v>135</v>
+      </c>
+      <c r="E9" s="0" t="s">
+        <v>181</v>
+      </c>
+      <c r="F9" s="0" t="s">
+        <v>182</v>
+      </c>
+      <c r="G9" s="5">
+        <v>3</v>
+      </c>
+      <c r="H9" s="5">
+        <v>2</v>
+      </c>
+      <c r="I9" s="5">
+        <v>2</v>
+      </c>
+      <c r="J9" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="K9" s="0" t="s">
+        <v>128</v>
+      </c>
+      <c r="L9" s="0" t="s">
+        <v>183</v>
+      </c>
+      <c r="M9" s="0" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="10" ht="20">
+      <c r="A10" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="D10" s="0" t="s">
+        <v>117</v>
+      </c>
+      <c r="E10" s="0" t="s">
+        <v>181</v>
+      </c>
+      <c r="F10" s="0" t="s">
+        <v>182</v>
+      </c>
+      <c r="G10" s="5">
+        <v>3</v>
+      </c>
+      <c r="H10" s="5">
+        <v>2</v>
+      </c>
+      <c r="I10" s="5">
+        <v>4</v>
+      </c>
+      <c r="J10" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="K10" s="0" t="s">
+        <v>139</v>
+      </c>
+      <c r="L10" s="0" t="s">
+        <v>183</v>
+      </c>
+      <c r="M10" s="0" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="11" ht="20">
+      <c r="A11" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="D11" s="0" t="s">
+        <v>132</v>
+      </c>
+      <c r="E11" s="0" t="s">
+        <v>181</v>
+      </c>
+      <c r="F11" s="0" t="s">
+        <v>182</v>
+      </c>
+      <c r="G11" s="5">
+        <v>2</v>
+      </c>
+      <c r="H11" s="5">
+        <v>2</v>
+      </c>
+      <c r="I11" s="5">
+        <v>4</v>
+      </c>
+      <c r="J11" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="K11" s="0" t="s">
+        <v>124</v>
+      </c>
+      <c r="L11" s="0" t="s">
+        <v>183</v>
+      </c>
+      <c r="M11" s="0" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="12" ht="20">
+      <c r="A12" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="D12" s="0" t="s">
+        <v>132</v>
+      </c>
+      <c r="E12" s="0" t="s">
+        <v>181</v>
+      </c>
+      <c r="F12" s="0" t="s">
+        <v>182</v>
+      </c>
+      <c r="G12" s="5">
+        <v>2</v>
+      </c>
+      <c r="H12" s="5">
+        <v>2</v>
+      </c>
+      <c r="I12" s="5">
+        <v>2</v>
+      </c>
+      <c r="J12" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="K12" s="0" t="s">
+        <v>128</v>
+      </c>
+      <c r="L12" s="0" t="s">
+        <v>183</v>
+      </c>
+      <c r="M12" s="0" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="13" ht="20">
+      <c r="A13" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="D13" s="0" t="s">
+        <v>132</v>
+      </c>
+      <c r="E13" s="0" t="s">
+        <v>181</v>
+      </c>
+      <c r="F13" s="0" t="s">
+        <v>182</v>
+      </c>
+      <c r="G13" s="5">
+        <v>2</v>
+      </c>
+      <c r="H13" s="5">
+        <v>2</v>
+      </c>
+      <c r="I13" s="5">
+        <v>4</v>
+      </c>
+      <c r="J13" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="K13" s="0" t="s">
+        <v>124</v>
+      </c>
+      <c r="L13" s="0" t="s">
+        <v>183</v>
+      </c>
+      <c r="M13" s="0" t="s">
+        <v>142</v>
       </c>
     </row>
   </sheetData>

</xml_diff>